<commit_message>
chore(templates): atualizar modelos NIS2 (revisao pos-validacao)
- registo-riscos.xlsx   17430 -> 17563 bytes
- inventario-ativos.xlsx 20299 -> 20476 bytes
- psi-template.docx     23305 -> 23285 bytes

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/assets/templates/inventario-ativos.xlsx
+++ b/backend/assets/templates/inventario-ativos.xlsx
@@ -42,49 +42,49 @@
     <t xml:space="preserve">📋  SEPARADORES DISPONÍVEIS</t>
   </si>
   <si>
-    <t xml:space="preserve">🖥  HARDWARE — Servidores, computadores, portáteis, equipamentos de rede, impressoras, dispositivos móveis</t>
-  </si>
-  <si>
-    <t xml:space="preserve">💾  SOFTWARE — Sistemas operativos, aplicações críticas, bases de dados, licenças</t>
-  </si>
-  <si>
-    <t xml:space="preserve">☁️  CLOUD E SAAS — Todos os serviços cloud contratados (M365, Google Workspace, ERP cloud, CRM, etc.)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">🌐  SUPERFÍCIE EXTERNA — Ativos expostos à Internet detetados pelo scanner CISPLAN (domínios, IPs, serviços, versões)</t>
+    <t xml:space="preserve">🌐  SUPERFÍCIE EXTERNA  ✅ AUTOMÁTICO — Ativos expostos à Internet, preenchidos pelo scanner CISPLAN (domínios, portos, serviços, versões). Reveja e classifique a criticidade.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">🖥  HARDWARE  ✏️ MANUAL — Servidores, computadores, portáteis, equipamentos de rede, impressoras. Preenchido pela empresa.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">💾  SOFTWARE  ✏️ MANUAL — Sistemas operativos, aplicações críticas, bases de dados, licenças. Preenchido pela empresa.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">☁️  CLOUD E SAAS  ✏️ MANUAL — Serviços cloud contratados (M365, Google Workspace, etc.). Preenchido pela empresa.</t>
   </si>
   <si>
     <t xml:space="preserve">⚠️  CLASSIFICAÇÃO DE CRITICIDADE</t>
   </si>
   <si>
-    <t xml:space="preserve">🔴  CRÍTICO — Se este ativo ficar indisponível ou comprometido, a empresa para ou sofre dano grave irreversível</t>
-  </si>
-  <si>
-    <t xml:space="preserve">🟠  ALTO — Impacto operacional significativo mas a empresa consegue operar em modo degradado por tempo limitado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">🟡  MÉDIO — Inconveniente operacional relevante mas impacto limitado e controlável</t>
-  </si>
-  <si>
-    <t xml:space="preserve">⚪  BAIXO — Impacto mínimo. A empresa funciona normalmente sem este ativo por períodos alargados</t>
-  </si>
-  <si>
-    <t xml:space="preserve">📚  INSTRUÇÕES DE PREENCHIMENTO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Preencha todos os campos — as células com fundo AMARELO são obrigatórias para conformidade NIS2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2. Use os menus dropdown nas colunas de Criticidade e Estado para garantir consistência</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3. Atribua um RESPONSÁVEL nomeado a cada ativo crítico — não use 'Departamento de TI' genérico</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4. Reveja e atualize este inventário quando: adquirir novos ativos, alterar fornecedores cloud, mudar colaboradores-chave</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5. Este documento é EVIDÊNCIA para auditoria CNCS — mantenha a data de última atualização sempre atual</t>
+    <t xml:space="preserve">CRÍTICO — Se este ativo ficar indisponível ou comprometido, a empresa PARA ou sofre dano grave (financeiro, legal ou reputacional)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ALTO — Impacto operacional significativo mas a empresa consegue operar em modo degradado por tempo limitado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MÉDIO — Inconveniente operacional relevante mas impacto limitado e controlável</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BAIXO — Impacto mínimo. A empresa funciona normalmente sem este ativo por períodos alargados</t>
+  </si>
+  <si>
+    <t xml:space="preserve">📚  COMO USAR ESTE DOCUMENTO PRÉ-PREENCHIDO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. O separador SUPERFÍCIE EXTERNA já vem preenchido com os ativos que o scanner CISPLAN detetou expostos à Internet — reveja-os e defina a criticidade de cada um</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. Preencha os separadores HARDWARE, SOFTWARE e CLOUD E SAAS com o inventário interno da empresa (equipamentos, aplicações e serviços que o scanner não vê de fora)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. Atribua um RESPONSÁVEL nomeado a cada ativo crítico — não use 'Departamento de TI', use o nome da pessoa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. Reveja e atualize quando adquirir novos ativos, alterar infraestrutura, ou pelo menos 1×/ano (obrigação NIS2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5. Este documento é EVIDÊNCIA para auditoria CNCS — mantenha a data de última atualização visível</t>
   </si>
   <si>
     <t xml:space="preserve">Versão 1.0 — 2025  |  NIS2 para PMEs em Portugal  |  Baseado em ISO/IEC 27001:2022 Controlo 5.9</t>
@@ -850,7 +850,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="45">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -887,19 +887,19 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -915,6 +915,10 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="14" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="15" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -927,16 +931,8 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="14" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="16" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -1490,19 +1486,45 @@
       <c r="B2" s="9" t="s">
         <v>22</v>
       </c>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
+      <c r="I2" s="9"/>
+      <c r="J2" s="9"/>
+      <c r="K2" s="9"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="10" t="s">
         <v>23</v>
       </c>
+      <c r="C3" s="10"/>
+      <c r="D3" s="10"/>
+      <c r="E3" s="10"/>
       <c r="F3" s="11" t="s">
         <v>24</v>
       </c>
+      <c r="G3" s="11"/>
+      <c r="H3" s="11"/>
+      <c r="I3" s="11"/>
+      <c r="J3" s="11"/>
+      <c r="K3" s="11"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="12" t="s">
         <v>25</v>
       </c>
+      <c r="C4" s="12"/>
+      <c r="D4" s="12"/>
+      <c r="E4" s="12"/>
+      <c r="F4" s="12"/>
+      <c r="G4" s="12"/>
+      <c r="H4" s="12"/>
+      <c r="I4" s="12"/>
+      <c r="J4" s="12"/>
+      <c r="K4" s="12"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="13" t="s">
@@ -1545,24 +1567,24 @@
       <c r="E6" s="15"/>
       <c r="F6" s="15"/>
       <c r="G6" s="15"/>
-      <c r="H6" s="15"/>
-      <c r="I6" s="16"/>
+      <c r="H6" s="16"/>
+      <c r="I6" s="17"/>
       <c r="J6" s="15"/>
       <c r="K6" s="15"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B7" s="17" t="s">
+      <c r="B7" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="C7" s="18"/>
-      <c r="D7" s="18"/>
-      <c r="E7" s="18"/>
-      <c r="F7" s="18"/>
-      <c r="G7" s="18"/>
-      <c r="H7" s="18"/>
-      <c r="I7" s="16"/>
-      <c r="J7" s="18"/>
-      <c r="K7" s="18"/>
+      <c r="C7" s="19"/>
+      <c r="D7" s="19"/>
+      <c r="E7" s="19"/>
+      <c r="F7" s="19"/>
+      <c r="G7" s="19"/>
+      <c r="H7" s="20"/>
+      <c r="I7" s="17"/>
+      <c r="J7" s="19"/>
+      <c r="K7" s="19"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="14" t="s">
@@ -1573,24 +1595,24 @@
       <c r="E8" s="15"/>
       <c r="F8" s="15"/>
       <c r="G8" s="15"/>
-      <c r="H8" s="15"/>
-      <c r="I8" s="16"/>
+      <c r="H8" s="16"/>
+      <c r="I8" s="17"/>
       <c r="J8" s="15"/>
       <c r="K8" s="15"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B9" s="17" t="s">
+      <c r="B9" s="18" t="s">
         <v>39</v>
       </c>
-      <c r="C9" s="18"/>
-      <c r="D9" s="18"/>
-      <c r="E9" s="18"/>
-      <c r="F9" s="18"/>
-      <c r="G9" s="18"/>
-      <c r="H9" s="18"/>
-      <c r="I9" s="16"/>
-      <c r="J9" s="18"/>
-      <c r="K9" s="18"/>
+      <c r="C9" s="19"/>
+      <c r="D9" s="19"/>
+      <c r="E9" s="19"/>
+      <c r="F9" s="19"/>
+      <c r="G9" s="19"/>
+      <c r="H9" s="20"/>
+      <c r="I9" s="17"/>
+      <c r="J9" s="19"/>
+      <c r="K9" s="19"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="14" t="s">
@@ -1601,24 +1623,24 @@
       <c r="E10" s="15"/>
       <c r="F10" s="15"/>
       <c r="G10" s="15"/>
-      <c r="H10" s="15"/>
-      <c r="I10" s="16"/>
+      <c r="H10" s="16"/>
+      <c r="I10" s="17"/>
       <c r="J10" s="15"/>
       <c r="K10" s="15"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B11" s="17" t="s">
+      <c r="B11" s="18" t="s">
         <v>41</v>
       </c>
-      <c r="C11" s="18"/>
-      <c r="D11" s="18"/>
-      <c r="E11" s="18"/>
-      <c r="F11" s="18"/>
-      <c r="G11" s="18"/>
-      <c r="H11" s="18"/>
-      <c r="I11" s="16"/>
-      <c r="J11" s="18"/>
-      <c r="K11" s="18"/>
+      <c r="C11" s="19"/>
+      <c r="D11" s="19"/>
+      <c r="E11" s="19"/>
+      <c r="F11" s="19"/>
+      <c r="G11" s="19"/>
+      <c r="H11" s="20"/>
+      <c r="I11" s="17"/>
+      <c r="J11" s="19"/>
+      <c r="K11" s="19"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="14" t="s">
@@ -1629,24 +1651,24 @@
       <c r="E12" s="15"/>
       <c r="F12" s="15"/>
       <c r="G12" s="15"/>
-      <c r="H12" s="15"/>
-      <c r="I12" s="16"/>
+      <c r="H12" s="16"/>
+      <c r="I12" s="17"/>
       <c r="J12" s="15"/>
       <c r="K12" s="15"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B13" s="17" t="s">
+      <c r="B13" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="C13" s="18"/>
-      <c r="D13" s="18"/>
-      <c r="E13" s="18"/>
-      <c r="F13" s="18"/>
-      <c r="G13" s="18"/>
-      <c r="H13" s="18"/>
-      <c r="I13" s="16"/>
-      <c r="J13" s="18"/>
-      <c r="K13" s="18"/>
+      <c r="C13" s="19"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="19"/>
+      <c r="F13" s="19"/>
+      <c r="G13" s="19"/>
+      <c r="H13" s="20"/>
+      <c r="I13" s="17"/>
+      <c r="J13" s="19"/>
+      <c r="K13" s="19"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B14" s="14" t="s">
@@ -1657,24 +1679,24 @@
       <c r="E14" s="15"/>
       <c r="F14" s="15"/>
       <c r="G14" s="15"/>
-      <c r="H14" s="15"/>
-      <c r="I14" s="16"/>
+      <c r="H14" s="16"/>
+      <c r="I14" s="17"/>
       <c r="J14" s="15"/>
       <c r="K14" s="15"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B15" s="17" t="s">
+      <c r="B15" s="18" t="s">
         <v>45</v>
       </c>
-      <c r="C15" s="18"/>
-      <c r="D15" s="18"/>
-      <c r="E15" s="18"/>
-      <c r="F15" s="18"/>
-      <c r="G15" s="18"/>
-      <c r="H15" s="18"/>
-      <c r="I15" s="16"/>
-      <c r="J15" s="18"/>
-      <c r="K15" s="18"/>
+      <c r="C15" s="19"/>
+      <c r="D15" s="19"/>
+      <c r="E15" s="19"/>
+      <c r="F15" s="19"/>
+      <c r="G15" s="19"/>
+      <c r="H15" s="20"/>
+      <c r="I15" s="17"/>
+      <c r="J15" s="19"/>
+      <c r="K15" s="19"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="14" t="s">
@@ -1685,24 +1707,24 @@
       <c r="E16" s="15"/>
       <c r="F16" s="15"/>
       <c r="G16" s="15"/>
-      <c r="H16" s="15"/>
-      <c r="I16" s="16"/>
+      <c r="H16" s="16"/>
+      <c r="I16" s="17"/>
       <c r="J16" s="15"/>
       <c r="K16" s="15"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B17" s="17" t="s">
+      <c r="B17" s="18" t="s">
         <v>47</v>
       </c>
-      <c r="C17" s="18"/>
-      <c r="D17" s="18"/>
-      <c r="E17" s="18"/>
-      <c r="F17" s="18"/>
-      <c r="G17" s="18"/>
-      <c r="H17" s="18"/>
-      <c r="I17" s="16"/>
-      <c r="J17" s="18"/>
-      <c r="K17" s="18"/>
+      <c r="C17" s="19"/>
+      <c r="D17" s="19"/>
+      <c r="E17" s="19"/>
+      <c r="F17" s="19"/>
+      <c r="G17" s="19"/>
+      <c r="H17" s="20"/>
+      <c r="I17" s="17"/>
+      <c r="J17" s="19"/>
+      <c r="K17" s="19"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B18" s="14" t="s">
@@ -1713,24 +1735,24 @@
       <c r="E18" s="15"/>
       <c r="F18" s="15"/>
       <c r="G18" s="15"/>
-      <c r="H18" s="15"/>
-      <c r="I18" s="16"/>
+      <c r="H18" s="16"/>
+      <c r="I18" s="17"/>
       <c r="J18" s="15"/>
       <c r="K18" s="15"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B19" s="17" t="s">
+      <c r="B19" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="C19" s="18"/>
-      <c r="D19" s="18"/>
-      <c r="E19" s="18"/>
-      <c r="F19" s="18"/>
-      <c r="G19" s="18"/>
-      <c r="H19" s="18"/>
-      <c r="I19" s="16"/>
-      <c r="J19" s="18"/>
-      <c r="K19" s="18"/>
+      <c r="C19" s="19"/>
+      <c r="D19" s="19"/>
+      <c r="E19" s="19"/>
+      <c r="F19" s="19"/>
+      <c r="G19" s="19"/>
+      <c r="H19" s="20"/>
+      <c r="I19" s="17"/>
+      <c r="J19" s="19"/>
+      <c r="K19" s="19"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B20" s="14" t="s">
@@ -1741,24 +1763,24 @@
       <c r="E20" s="15"/>
       <c r="F20" s="15"/>
       <c r="G20" s="15"/>
-      <c r="H20" s="15"/>
-      <c r="I20" s="16"/>
+      <c r="H20" s="16"/>
+      <c r="I20" s="17"/>
       <c r="J20" s="15"/>
       <c r="K20" s="15"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B21" s="17" t="s">
+      <c r="B21" s="18" t="s">
         <v>51</v>
       </c>
-      <c r="C21" s="18"/>
-      <c r="D21" s="18"/>
-      <c r="E21" s="18"/>
-      <c r="F21" s="18"/>
-      <c r="G21" s="18"/>
-      <c r="H21" s="18"/>
-      <c r="I21" s="16"/>
-      <c r="J21" s="18"/>
-      <c r="K21" s="18"/>
+      <c r="C21" s="19"/>
+      <c r="D21" s="19"/>
+      <c r="E21" s="19"/>
+      <c r="F21" s="19"/>
+      <c r="G21" s="19"/>
+      <c r="H21" s="20"/>
+      <c r="I21" s="17"/>
+      <c r="J21" s="19"/>
+      <c r="K21" s="19"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B22" s="14" t="s">
@@ -1769,26 +1791,32 @@
       <c r="E22" s="15"/>
       <c r="F22" s="15"/>
       <c r="G22" s="15"/>
-      <c r="H22" s="15"/>
-      <c r="I22" s="16"/>
+      <c r="H22" s="16"/>
+      <c r="I22" s="17"/>
       <c r="J22" s="15"/>
       <c r="K22" s="15"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B23" s="17" t="s">
+      <c r="B23" s="18" t="s">
         <v>53</v>
       </c>
-      <c r="C23" s="18"/>
-      <c r="D23" s="18"/>
-      <c r="E23" s="18"/>
-      <c r="F23" s="18"/>
-      <c r="G23" s="18"/>
-      <c r="H23" s="18"/>
-      <c r="I23" s="16"/>
-      <c r="J23" s="18"/>
-      <c r="K23" s="18"/>
+      <c r="C23" s="19"/>
+      <c r="D23" s="19"/>
+      <c r="E23" s="19"/>
+      <c r="F23" s="19"/>
+      <c r="G23" s="19"/>
+      <c r="H23" s="20"/>
+      <c r="I23" s="17"/>
+      <c r="J23" s="19"/>
+      <c r="K23" s="19"/>
     </row>
   </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="B2:K2"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="F3:K3"/>
+    <mergeCell ref="B4:K4"/>
+  </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -1820,34 +1848,34 @@
   </cols>
   <sheetData>
     <row r="2" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
-      <c r="I2" s="19"/>
-      <c r="J2" s="19"/>
-      <c r="K2" s="19"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
+      <c r="I2" s="9"/>
+      <c r="J2" s="9"/>
+      <c r="K2" s="9"/>
     </row>
     <row r="3" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B3" s="20" t="s">
+      <c r="B3" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
-      <c r="E3" s="20"/>
-      <c r="F3" s="21" t="s">
+      <c r="C3" s="10"/>
+      <c r="D3" s="10"/>
+      <c r="E3" s="10"/>
+      <c r="F3" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="G3" s="21"/>
-      <c r="H3" s="21"/>
-      <c r="I3" s="21"/>
-      <c r="J3" s="21"/>
-      <c r="K3" s="21"/>
+      <c r="G3" s="11"/>
+      <c r="H3" s="11"/>
+      <c r="I3" s="11"/>
+      <c r="J3" s="11"/>
+      <c r="K3" s="11"/>
     </row>
     <row r="5" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="13" t="s">
@@ -1891,23 +1919,23 @@
       <c r="F6" s="15"/>
       <c r="G6" s="15"/>
       <c r="H6" s="15"/>
-      <c r="I6" s="16"/>
+      <c r="I6" s="17"/>
       <c r="J6" s="15"/>
       <c r="K6" s="15"/>
     </row>
     <row r="7" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B7" s="17" t="s">
+      <c r="B7" s="18" t="s">
         <v>63</v>
       </c>
-      <c r="C7" s="18"/>
-      <c r="D7" s="18"/>
-      <c r="E7" s="18"/>
-      <c r="F7" s="18"/>
-      <c r="G7" s="18"/>
-      <c r="H7" s="18"/>
-      <c r="I7" s="16"/>
-      <c r="J7" s="18"/>
-      <c r="K7" s="18"/>
+      <c r="C7" s="19"/>
+      <c r="D7" s="19"/>
+      <c r="E7" s="19"/>
+      <c r="F7" s="19"/>
+      <c r="G7" s="19"/>
+      <c r="H7" s="19"/>
+      <c r="I7" s="17"/>
+      <c r="J7" s="19"/>
+      <c r="K7" s="19"/>
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="14" t="s">
@@ -1919,23 +1947,23 @@
       <c r="F8" s="15"/>
       <c r="G8" s="15"/>
       <c r="H8" s="15"/>
-      <c r="I8" s="16"/>
+      <c r="I8" s="17"/>
       <c r="J8" s="15"/>
       <c r="K8" s="15"/>
     </row>
     <row r="9" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B9" s="17" t="s">
+      <c r="B9" s="18" t="s">
         <v>65</v>
       </c>
-      <c r="C9" s="18"/>
-      <c r="D9" s="18"/>
-      <c r="E9" s="18"/>
-      <c r="F9" s="18"/>
-      <c r="G9" s="18"/>
-      <c r="H9" s="18"/>
-      <c r="I9" s="22"/>
-      <c r="J9" s="18"/>
-      <c r="K9" s="18"/>
+      <c r="C9" s="19"/>
+      <c r="D9" s="19"/>
+      <c r="E9" s="19"/>
+      <c r="F9" s="19"/>
+      <c r="G9" s="19"/>
+      <c r="H9" s="19"/>
+      <c r="I9" s="21"/>
+      <c r="J9" s="19"/>
+      <c r="K9" s="19"/>
     </row>
     <row r="10" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="14" t="s">
@@ -1947,23 +1975,23 @@
       <c r="F10" s="15"/>
       <c r="G10" s="15"/>
       <c r="H10" s="15"/>
-      <c r="I10" s="22"/>
+      <c r="I10" s="21"/>
       <c r="J10" s="15"/>
       <c r="K10" s="15"/>
     </row>
     <row r="11" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B11" s="17" t="s">
+      <c r="B11" s="18" t="s">
         <v>67</v>
       </c>
-      <c r="C11" s="18"/>
-      <c r="D11" s="18"/>
-      <c r="E11" s="18"/>
-      <c r="F11" s="18"/>
-      <c r="G11" s="18"/>
-      <c r="H11" s="18"/>
-      <c r="I11" s="16"/>
-      <c r="J11" s="18"/>
-      <c r="K11" s="18"/>
+      <c r="C11" s="19"/>
+      <c r="D11" s="19"/>
+      <c r="E11" s="19"/>
+      <c r="F11" s="19"/>
+      <c r="G11" s="19"/>
+      <c r="H11" s="19"/>
+      <c r="I11" s="17"/>
+      <c r="J11" s="19"/>
+      <c r="K11" s="19"/>
     </row>
     <row r="12" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="14" t="s">
@@ -1975,163 +2003,163 @@
       <c r="F12" s="15"/>
       <c r="G12" s="15"/>
       <c r="H12" s="15"/>
-      <c r="I12" s="22"/>
+      <c r="I12" s="21"/>
       <c r="J12" s="15"/>
       <c r="K12" s="15"/>
     </row>
     <row r="13" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B13" s="17" t="s">
+      <c r="B13" s="18" t="s">
         <v>69</v>
       </c>
-      <c r="C13" s="18"/>
-      <c r="D13" s="18"/>
-      <c r="E13" s="18"/>
-      <c r="F13" s="18"/>
-      <c r="G13" s="18"/>
-      <c r="H13" s="18"/>
-      <c r="I13" s="23"/>
-      <c r="J13" s="18"/>
-      <c r="K13" s="18"/>
+      <c r="C13" s="19"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="19"/>
+      <c r="F13" s="19"/>
+      <c r="G13" s="19"/>
+      <c r="H13" s="19"/>
+      <c r="I13" s="22"/>
+      <c r="J13" s="19"/>
+      <c r="K13" s="19"/>
     </row>
     <row r="14" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B14" s="24" t="s">
+      <c r="B14" s="23" t="s">
         <v>70</v>
       </c>
-      <c r="C14" s="25"/>
-      <c r="D14" s="25"/>
-      <c r="E14" s="25"/>
-      <c r="F14" s="25"/>
-      <c r="G14" s="25"/>
-      <c r="H14" s="25"/>
-      <c r="I14" s="26"/>
-      <c r="J14" s="25"/>
-      <c r="K14" s="25"/>
+      <c r="C14" s="24"/>
+      <c r="D14" s="24"/>
+      <c r="E14" s="24"/>
+      <c r="F14" s="24"/>
+      <c r="G14" s="24"/>
+      <c r="H14" s="24"/>
+      <c r="I14" s="25"/>
+      <c r="J14" s="24"/>
+      <c r="K14" s="24"/>
     </row>
     <row r="15" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B15" s="27" t="s">
+      <c r="B15" s="26" t="s">
         <v>71</v>
       </c>
-      <c r="C15" s="28"/>
-      <c r="D15" s="28"/>
-      <c r="E15" s="28"/>
-      <c r="F15" s="28"/>
-      <c r="G15" s="28"/>
-      <c r="H15" s="28"/>
-      <c r="I15" s="26"/>
-      <c r="J15" s="28"/>
-      <c r="K15" s="28"/>
+      <c r="C15" s="27"/>
+      <c r="D15" s="27"/>
+      <c r="E15" s="27"/>
+      <c r="F15" s="27"/>
+      <c r="G15" s="27"/>
+      <c r="H15" s="27"/>
+      <c r="I15" s="25"/>
+      <c r="J15" s="27"/>
+      <c r="K15" s="27"/>
     </row>
     <row r="16" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B16" s="24" t="s">
+      <c r="B16" s="23" t="s">
         <v>72</v>
       </c>
-      <c r="C16" s="25"/>
-      <c r="D16" s="25"/>
-      <c r="E16" s="25"/>
-      <c r="F16" s="25"/>
-      <c r="G16" s="25"/>
-      <c r="H16" s="25"/>
-      <c r="I16" s="26"/>
-      <c r="J16" s="25"/>
-      <c r="K16" s="25"/>
+      <c r="C16" s="24"/>
+      <c r="D16" s="24"/>
+      <c r="E16" s="24"/>
+      <c r="F16" s="24"/>
+      <c r="G16" s="24"/>
+      <c r="H16" s="24"/>
+      <c r="I16" s="25"/>
+      <c r="J16" s="24"/>
+      <c r="K16" s="24"/>
     </row>
     <row r="17" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B17" s="27" t="s">
+      <c r="B17" s="26" t="s">
         <v>73</v>
       </c>
-      <c r="C17" s="28"/>
-      <c r="D17" s="28"/>
-      <c r="E17" s="28"/>
-      <c r="F17" s="28"/>
-      <c r="G17" s="28"/>
-      <c r="H17" s="28"/>
-      <c r="I17" s="26"/>
-      <c r="J17" s="28"/>
-      <c r="K17" s="28"/>
+      <c r="C17" s="27"/>
+      <c r="D17" s="27"/>
+      <c r="E17" s="27"/>
+      <c r="F17" s="27"/>
+      <c r="G17" s="27"/>
+      <c r="H17" s="27"/>
+      <c r="I17" s="25"/>
+      <c r="J17" s="27"/>
+      <c r="K17" s="27"/>
     </row>
     <row r="18" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B18" s="24" t="s">
+      <c r="B18" s="23" t="s">
         <v>74</v>
       </c>
-      <c r="C18" s="25"/>
-      <c r="D18" s="25"/>
-      <c r="E18" s="25"/>
-      <c r="F18" s="25"/>
-      <c r="G18" s="25"/>
-      <c r="H18" s="25"/>
-      <c r="I18" s="26"/>
-      <c r="J18" s="25"/>
-      <c r="K18" s="25"/>
+      <c r="C18" s="24"/>
+      <c r="D18" s="24"/>
+      <c r="E18" s="24"/>
+      <c r="F18" s="24"/>
+      <c r="G18" s="24"/>
+      <c r="H18" s="24"/>
+      <c r="I18" s="25"/>
+      <c r="J18" s="24"/>
+      <c r="K18" s="24"/>
     </row>
     <row r="19" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B19" s="27" t="s">
+      <c r="B19" s="26" t="s">
         <v>75</v>
       </c>
-      <c r="C19" s="28"/>
-      <c r="D19" s="28"/>
-      <c r="E19" s="28"/>
-      <c r="F19" s="28"/>
-      <c r="G19" s="28"/>
-      <c r="H19" s="28"/>
-      <c r="I19" s="26"/>
-      <c r="J19" s="28"/>
-      <c r="K19" s="28"/>
+      <c r="C19" s="27"/>
+      <c r="D19" s="27"/>
+      <c r="E19" s="27"/>
+      <c r="F19" s="27"/>
+      <c r="G19" s="27"/>
+      <c r="H19" s="27"/>
+      <c r="I19" s="25"/>
+      <c r="J19" s="27"/>
+      <c r="K19" s="27"/>
     </row>
     <row r="20" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B20" s="24" t="s">
+      <c r="B20" s="23" t="s">
         <v>76</v>
       </c>
-      <c r="C20" s="25"/>
-      <c r="D20" s="25"/>
-      <c r="E20" s="25"/>
-      <c r="F20" s="25"/>
-      <c r="G20" s="25"/>
-      <c r="H20" s="25"/>
-      <c r="I20" s="26"/>
-      <c r="J20" s="25"/>
-      <c r="K20" s="25"/>
+      <c r="C20" s="24"/>
+      <c r="D20" s="24"/>
+      <c r="E20" s="24"/>
+      <c r="F20" s="24"/>
+      <c r="G20" s="24"/>
+      <c r="H20" s="24"/>
+      <c r="I20" s="25"/>
+      <c r="J20" s="24"/>
+      <c r="K20" s="24"/>
     </row>
     <row r="21" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B21" s="27" t="s">
+      <c r="B21" s="26" t="s">
         <v>77</v>
       </c>
-      <c r="C21" s="28"/>
-      <c r="D21" s="28"/>
-      <c r="E21" s="28"/>
-      <c r="F21" s="28"/>
-      <c r="G21" s="28"/>
-      <c r="H21" s="28"/>
-      <c r="I21" s="26"/>
-      <c r="J21" s="28"/>
-      <c r="K21" s="28"/>
+      <c r="C21" s="27"/>
+      <c r="D21" s="27"/>
+      <c r="E21" s="27"/>
+      <c r="F21" s="27"/>
+      <c r="G21" s="27"/>
+      <c r="H21" s="27"/>
+      <c r="I21" s="25"/>
+      <c r="J21" s="27"/>
+      <c r="K21" s="27"/>
     </row>
     <row r="22" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B22" s="24" t="s">
+      <c r="B22" s="23" t="s">
         <v>78</v>
       </c>
-      <c r="C22" s="25"/>
-      <c r="D22" s="25"/>
-      <c r="E22" s="25"/>
-      <c r="F22" s="25"/>
-      <c r="G22" s="25"/>
-      <c r="H22" s="25"/>
-      <c r="I22" s="26"/>
-      <c r="J22" s="25"/>
-      <c r="K22" s="25"/>
+      <c r="C22" s="24"/>
+      <c r="D22" s="24"/>
+      <c r="E22" s="24"/>
+      <c r="F22" s="24"/>
+      <c r="G22" s="24"/>
+      <c r="H22" s="24"/>
+      <c r="I22" s="25"/>
+      <c r="J22" s="24"/>
+      <c r="K22" s="24"/>
     </row>
     <row r="23" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B23" s="27" t="s">
+      <c r="B23" s="26" t="s">
         <v>79</v>
       </c>
-      <c r="C23" s="28"/>
-      <c r="D23" s="28"/>
-      <c r="E23" s="28"/>
-      <c r="F23" s="28"/>
-      <c r="G23" s="28"/>
-      <c r="H23" s="28"/>
-      <c r="I23" s="26"/>
-      <c r="J23" s="28"/>
-      <c r="K23" s="28"/>
+      <c r="C23" s="27"/>
+      <c r="D23" s="27"/>
+      <c r="E23" s="27"/>
+      <c r="F23" s="27"/>
+      <c r="G23" s="27"/>
+      <c r="H23" s="27"/>
+      <c r="I23" s="25"/>
+      <c r="J23" s="27"/>
+      <c r="K23" s="27"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -2170,34 +2198,34 @@
   </cols>
   <sheetData>
     <row r="2" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
-      <c r="I2" s="19"/>
-      <c r="J2" s="19"/>
-      <c r="K2" s="19"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
+      <c r="I2" s="9"/>
+      <c r="J2" s="9"/>
+      <c r="K2" s="9"/>
     </row>
     <row r="3" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B3" s="20" t="s">
+      <c r="B3" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
-      <c r="E3" s="20"/>
-      <c r="F3" s="21" t="s">
+      <c r="C3" s="10"/>
+      <c r="D3" s="10"/>
+      <c r="E3" s="10"/>
+      <c r="F3" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="G3" s="21"/>
-      <c r="H3" s="21"/>
-      <c r="I3" s="21"/>
-      <c r="J3" s="21"/>
-      <c r="K3" s="21"/>
+      <c r="G3" s="11"/>
+      <c r="H3" s="11"/>
+      <c r="I3" s="11"/>
+      <c r="J3" s="11"/>
+      <c r="K3" s="11"/>
     </row>
     <row r="5" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="13" t="s">
@@ -2241,23 +2269,23 @@
       <c r="F6" s="15"/>
       <c r="G6" s="15"/>
       <c r="H6" s="15"/>
-      <c r="I6" s="16"/>
+      <c r="I6" s="17"/>
       <c r="J6" s="15"/>
       <c r="K6" s="15"/>
     </row>
     <row r="7" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B7" s="17" t="s">
+      <c r="B7" s="18" t="s">
         <v>89</v>
       </c>
-      <c r="C7" s="18"/>
-      <c r="D7" s="18"/>
-      <c r="E7" s="18"/>
-      <c r="F7" s="18"/>
-      <c r="G7" s="18"/>
-      <c r="H7" s="18"/>
-      <c r="I7" s="16"/>
-      <c r="J7" s="18"/>
-      <c r="K7" s="18"/>
+      <c r="C7" s="19"/>
+      <c r="D7" s="19"/>
+      <c r="E7" s="19"/>
+      <c r="F7" s="19"/>
+      <c r="G7" s="19"/>
+      <c r="H7" s="19"/>
+      <c r="I7" s="17"/>
+      <c r="J7" s="19"/>
+      <c r="K7" s="19"/>
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="14" t="s">
@@ -2269,23 +2297,23 @@
       <c r="F8" s="15"/>
       <c r="G8" s="15"/>
       <c r="H8" s="15"/>
-      <c r="I8" s="16"/>
+      <c r="I8" s="17"/>
       <c r="J8" s="15"/>
       <c r="K8" s="15"/>
     </row>
     <row r="9" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B9" s="17" t="s">
+      <c r="B9" s="18" t="s">
         <v>91</v>
       </c>
-      <c r="C9" s="18"/>
-      <c r="D9" s="18"/>
-      <c r="E9" s="18"/>
-      <c r="F9" s="18"/>
-      <c r="G9" s="18"/>
-      <c r="H9" s="18"/>
-      <c r="I9" s="16"/>
-      <c r="J9" s="18"/>
-      <c r="K9" s="18"/>
+      <c r="C9" s="19"/>
+      <c r="D9" s="19"/>
+      <c r="E9" s="19"/>
+      <c r="F9" s="19"/>
+      <c r="G9" s="19"/>
+      <c r="H9" s="19"/>
+      <c r="I9" s="17"/>
+      <c r="J9" s="19"/>
+      <c r="K9" s="19"/>
     </row>
     <row r="10" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="14" t="s">
@@ -2297,23 +2325,23 @@
       <c r="F10" s="15"/>
       <c r="G10" s="15"/>
       <c r="H10" s="15"/>
-      <c r="I10" s="22"/>
+      <c r="I10" s="21"/>
       <c r="J10" s="15"/>
       <c r="K10" s="15"/>
     </row>
     <row r="11" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B11" s="17" t="s">
+      <c r="B11" s="18" t="s">
         <v>93</v>
       </c>
-      <c r="C11" s="18"/>
-      <c r="D11" s="18"/>
-      <c r="E11" s="18"/>
-      <c r="F11" s="18"/>
-      <c r="G11" s="18"/>
-      <c r="H11" s="18"/>
-      <c r="I11" s="16"/>
-      <c r="J11" s="18"/>
-      <c r="K11" s="18"/>
+      <c r="C11" s="19"/>
+      <c r="D11" s="19"/>
+      <c r="E11" s="19"/>
+      <c r="F11" s="19"/>
+      <c r="G11" s="19"/>
+      <c r="H11" s="19"/>
+      <c r="I11" s="17"/>
+      <c r="J11" s="19"/>
+      <c r="K11" s="19"/>
     </row>
     <row r="12" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="14" t="s">
@@ -2325,163 +2353,163 @@
       <c r="F12" s="15"/>
       <c r="G12" s="15"/>
       <c r="H12" s="15"/>
-      <c r="I12" s="23"/>
+      <c r="I12" s="22"/>
       <c r="J12" s="15"/>
       <c r="K12" s="15"/>
     </row>
     <row r="13" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B13" s="17" t="s">
+      <c r="B13" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="C13" s="18"/>
-      <c r="D13" s="18"/>
-      <c r="E13" s="18"/>
-      <c r="F13" s="18"/>
-      <c r="G13" s="18"/>
-      <c r="H13" s="18"/>
-      <c r="I13" s="22"/>
-      <c r="J13" s="18"/>
-      <c r="K13" s="18"/>
+      <c r="C13" s="19"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="19"/>
+      <c r="F13" s="19"/>
+      <c r="G13" s="19"/>
+      <c r="H13" s="19"/>
+      <c r="I13" s="21"/>
+      <c r="J13" s="19"/>
+      <c r="K13" s="19"/>
     </row>
     <row r="14" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B14" s="24" t="s">
+      <c r="B14" s="23" t="s">
         <v>96</v>
       </c>
-      <c r="C14" s="25"/>
-      <c r="D14" s="25"/>
-      <c r="E14" s="25"/>
-      <c r="F14" s="25"/>
-      <c r="G14" s="25"/>
-      <c r="H14" s="25"/>
-      <c r="I14" s="26"/>
-      <c r="J14" s="25"/>
-      <c r="K14" s="25"/>
+      <c r="C14" s="24"/>
+      <c r="D14" s="24"/>
+      <c r="E14" s="24"/>
+      <c r="F14" s="24"/>
+      <c r="G14" s="24"/>
+      <c r="H14" s="24"/>
+      <c r="I14" s="25"/>
+      <c r="J14" s="24"/>
+      <c r="K14" s="24"/>
     </row>
     <row r="15" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B15" s="27" t="s">
+      <c r="B15" s="26" t="s">
         <v>97</v>
       </c>
-      <c r="C15" s="28"/>
-      <c r="D15" s="28"/>
-      <c r="E15" s="28"/>
-      <c r="F15" s="28"/>
-      <c r="G15" s="28"/>
-      <c r="H15" s="28"/>
-      <c r="I15" s="26"/>
-      <c r="J15" s="28"/>
-      <c r="K15" s="28"/>
+      <c r="C15" s="27"/>
+      <c r="D15" s="27"/>
+      <c r="E15" s="27"/>
+      <c r="F15" s="27"/>
+      <c r="G15" s="27"/>
+      <c r="H15" s="27"/>
+      <c r="I15" s="25"/>
+      <c r="J15" s="27"/>
+      <c r="K15" s="27"/>
     </row>
     <row r="16" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B16" s="24" t="s">
+      <c r="B16" s="23" t="s">
         <v>98</v>
       </c>
-      <c r="C16" s="25"/>
-      <c r="D16" s="25"/>
-      <c r="E16" s="25"/>
-      <c r="F16" s="25"/>
-      <c r="G16" s="25"/>
-      <c r="H16" s="25"/>
-      <c r="I16" s="26"/>
-      <c r="J16" s="25"/>
-      <c r="K16" s="25"/>
+      <c r="C16" s="24"/>
+      <c r="D16" s="24"/>
+      <c r="E16" s="24"/>
+      <c r="F16" s="24"/>
+      <c r="G16" s="24"/>
+      <c r="H16" s="24"/>
+      <c r="I16" s="25"/>
+      <c r="J16" s="24"/>
+      <c r="K16" s="24"/>
     </row>
     <row r="17" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B17" s="27" t="s">
+      <c r="B17" s="26" t="s">
         <v>99</v>
       </c>
-      <c r="C17" s="28"/>
-      <c r="D17" s="28"/>
-      <c r="E17" s="28"/>
-      <c r="F17" s="28"/>
-      <c r="G17" s="28"/>
-      <c r="H17" s="28"/>
-      <c r="I17" s="26"/>
-      <c r="J17" s="28"/>
-      <c r="K17" s="28"/>
+      <c r="C17" s="27"/>
+      <c r="D17" s="27"/>
+      <c r="E17" s="27"/>
+      <c r="F17" s="27"/>
+      <c r="G17" s="27"/>
+      <c r="H17" s="27"/>
+      <c r="I17" s="25"/>
+      <c r="J17" s="27"/>
+      <c r="K17" s="27"/>
     </row>
     <row r="18" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B18" s="24" t="s">
+      <c r="B18" s="23" t="s">
         <v>100</v>
       </c>
-      <c r="C18" s="25"/>
-      <c r="D18" s="25"/>
-      <c r="E18" s="25"/>
-      <c r="F18" s="25"/>
-      <c r="G18" s="25"/>
-      <c r="H18" s="25"/>
-      <c r="I18" s="26"/>
-      <c r="J18" s="25"/>
-      <c r="K18" s="25"/>
+      <c r="C18" s="24"/>
+      <c r="D18" s="24"/>
+      <c r="E18" s="24"/>
+      <c r="F18" s="24"/>
+      <c r="G18" s="24"/>
+      <c r="H18" s="24"/>
+      <c r="I18" s="25"/>
+      <c r="J18" s="24"/>
+      <c r="K18" s="24"/>
     </row>
     <row r="19" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B19" s="27" t="s">
+      <c r="B19" s="26" t="s">
         <v>101</v>
       </c>
-      <c r="C19" s="28"/>
-      <c r="D19" s="28"/>
-      <c r="E19" s="28"/>
-      <c r="F19" s="28"/>
-      <c r="G19" s="28"/>
-      <c r="H19" s="28"/>
-      <c r="I19" s="26"/>
-      <c r="J19" s="28"/>
-      <c r="K19" s="28"/>
+      <c r="C19" s="27"/>
+      <c r="D19" s="27"/>
+      <c r="E19" s="27"/>
+      <c r="F19" s="27"/>
+      <c r="G19" s="27"/>
+      <c r="H19" s="27"/>
+      <c r="I19" s="25"/>
+      <c r="J19" s="27"/>
+      <c r="K19" s="27"/>
     </row>
     <row r="20" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B20" s="24" t="s">
+      <c r="B20" s="23" t="s">
         <v>102</v>
       </c>
-      <c r="C20" s="25"/>
-      <c r="D20" s="25"/>
-      <c r="E20" s="25"/>
-      <c r="F20" s="25"/>
-      <c r="G20" s="25"/>
-      <c r="H20" s="25"/>
-      <c r="I20" s="26"/>
-      <c r="J20" s="25"/>
-      <c r="K20" s="25"/>
+      <c r="C20" s="24"/>
+      <c r="D20" s="24"/>
+      <c r="E20" s="24"/>
+      <c r="F20" s="24"/>
+      <c r="G20" s="24"/>
+      <c r="H20" s="24"/>
+      <c r="I20" s="25"/>
+      <c r="J20" s="24"/>
+      <c r="K20" s="24"/>
     </row>
     <row r="21" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B21" s="27" t="s">
+      <c r="B21" s="26" t="s">
         <v>103</v>
       </c>
-      <c r="C21" s="28"/>
-      <c r="D21" s="28"/>
-      <c r="E21" s="28"/>
-      <c r="F21" s="28"/>
-      <c r="G21" s="28"/>
-      <c r="H21" s="28"/>
-      <c r="I21" s="26"/>
-      <c r="J21" s="28"/>
-      <c r="K21" s="28"/>
+      <c r="C21" s="27"/>
+      <c r="D21" s="27"/>
+      <c r="E21" s="27"/>
+      <c r="F21" s="27"/>
+      <c r="G21" s="27"/>
+      <c r="H21" s="27"/>
+      <c r="I21" s="25"/>
+      <c r="J21" s="27"/>
+      <c r="K21" s="27"/>
     </row>
     <row r="22" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B22" s="24" t="s">
+      <c r="B22" s="23" t="s">
         <v>104</v>
       </c>
-      <c r="C22" s="25"/>
-      <c r="D22" s="25"/>
-      <c r="E22" s="25"/>
-      <c r="F22" s="25"/>
-      <c r="G22" s="25"/>
-      <c r="H22" s="25"/>
-      <c r="I22" s="26"/>
-      <c r="J22" s="25"/>
-      <c r="K22" s="25"/>
+      <c r="C22" s="24"/>
+      <c r="D22" s="24"/>
+      <c r="E22" s="24"/>
+      <c r="F22" s="24"/>
+      <c r="G22" s="24"/>
+      <c r="H22" s="24"/>
+      <c r="I22" s="25"/>
+      <c r="J22" s="24"/>
+      <c r="K22" s="24"/>
     </row>
     <row r="23" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B23" s="27" t="s">
+      <c r="B23" s="26" t="s">
         <v>105</v>
       </c>
-      <c r="C23" s="28"/>
-      <c r="D23" s="28"/>
-      <c r="E23" s="28"/>
-      <c r="F23" s="28"/>
-      <c r="G23" s="28"/>
-      <c r="H23" s="28"/>
-      <c r="I23" s="26"/>
-      <c r="J23" s="28"/>
-      <c r="K23" s="28"/>
+      <c r="C23" s="27"/>
+      <c r="D23" s="27"/>
+      <c r="E23" s="27"/>
+      <c r="F23" s="27"/>
+      <c r="G23" s="27"/>
+      <c r="H23" s="27"/>
+      <c r="I23" s="25"/>
+      <c r="J23" s="27"/>
+      <c r="K23" s="27"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -2519,34 +2547,34 @@
   </cols>
   <sheetData>
     <row r="2" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
-      <c r="I2" s="19"/>
-      <c r="J2" s="19"/>
-      <c r="K2" s="19"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
+      <c r="I2" s="9"/>
+      <c r="J2" s="9"/>
+      <c r="K2" s="9"/>
     </row>
     <row r="3" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B3" s="29" t="s">
+      <c r="B3" s="28" t="s">
         <v>23</v>
       </c>
-      <c r="C3" s="29"/>
-      <c r="D3" s="29"/>
-      <c r="E3" s="29"/>
-      <c r="F3" s="30" t="s">
+      <c r="C3" s="28"/>
+      <c r="D3" s="28"/>
+      <c r="E3" s="28"/>
+      <c r="F3" s="29" t="s">
         <v>55</v>
       </c>
-      <c r="G3" s="30"/>
-      <c r="H3" s="30"/>
-      <c r="I3" s="30"/>
-      <c r="J3" s="30"/>
-      <c r="K3" s="30"/>
+      <c r="G3" s="29"/>
+      <c r="H3" s="29"/>
+      <c r="I3" s="29"/>
+      <c r="J3" s="29"/>
+      <c r="K3" s="29"/>
     </row>
     <row r="5" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="13" t="s">
@@ -2590,23 +2618,23 @@
       <c r="F6" s="15"/>
       <c r="G6" s="15"/>
       <c r="H6" s="15"/>
-      <c r="I6" s="16"/>
+      <c r="I6" s="17"/>
       <c r="J6" s="15"/>
-      <c r="K6" s="31"/>
+      <c r="K6" s="30"/>
     </row>
     <row r="7" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B7" s="17" t="s">
+      <c r="B7" s="18" t="s">
         <v>115</v>
       </c>
-      <c r="C7" s="18"/>
-      <c r="D7" s="18"/>
-      <c r="E7" s="18"/>
-      <c r="F7" s="18"/>
-      <c r="G7" s="18"/>
-      <c r="H7" s="18"/>
-      <c r="I7" s="16"/>
-      <c r="J7" s="18"/>
-      <c r="K7" s="31"/>
+      <c r="C7" s="19"/>
+      <c r="D7" s="19"/>
+      <c r="E7" s="19"/>
+      <c r="F7" s="19"/>
+      <c r="G7" s="19"/>
+      <c r="H7" s="19"/>
+      <c r="I7" s="17"/>
+      <c r="J7" s="19"/>
+      <c r="K7" s="30"/>
     </row>
     <row r="8" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="14" t="s">
@@ -2618,23 +2646,23 @@
       <c r="F8" s="15"/>
       <c r="G8" s="15"/>
       <c r="H8" s="15"/>
-      <c r="I8" s="16"/>
+      <c r="I8" s="17"/>
       <c r="J8" s="15"/>
-      <c r="K8" s="32"/>
+      <c r="K8" s="31"/>
     </row>
     <row r="9" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B9" s="17" t="s">
+      <c r="B9" s="18" t="s">
         <v>117</v>
       </c>
-      <c r="C9" s="18"/>
-      <c r="D9" s="18"/>
-      <c r="E9" s="18"/>
-      <c r="F9" s="18"/>
-      <c r="G9" s="18"/>
-      <c r="H9" s="18"/>
-      <c r="I9" s="16"/>
-      <c r="J9" s="18"/>
-      <c r="K9" s="32"/>
+      <c r="C9" s="19"/>
+      <c r="D9" s="19"/>
+      <c r="E9" s="19"/>
+      <c r="F9" s="19"/>
+      <c r="G9" s="19"/>
+      <c r="H9" s="19"/>
+      <c r="I9" s="17"/>
+      <c r="J9" s="19"/>
+      <c r="K9" s="31"/>
     </row>
     <row r="10" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="14" t="s">
@@ -2646,23 +2674,23 @@
       <c r="F10" s="15"/>
       <c r="G10" s="15"/>
       <c r="H10" s="15"/>
-      <c r="I10" s="16"/>
+      <c r="I10" s="17"/>
       <c r="J10" s="15"/>
-      <c r="K10" s="33"/>
+      <c r="K10" s="32"/>
     </row>
     <row r="11" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B11" s="17" t="s">
+      <c r="B11" s="18" t="s">
         <v>119</v>
       </c>
-      <c r="C11" s="18"/>
-      <c r="D11" s="18"/>
-      <c r="E11" s="18"/>
-      <c r="F11" s="18"/>
-      <c r="G11" s="18"/>
-      <c r="H11" s="18"/>
-      <c r="I11" s="22"/>
-      <c r="J11" s="18"/>
-      <c r="K11" s="32"/>
+      <c r="C11" s="19"/>
+      <c r="D11" s="19"/>
+      <c r="E11" s="19"/>
+      <c r="F11" s="19"/>
+      <c r="G11" s="19"/>
+      <c r="H11" s="19"/>
+      <c r="I11" s="21"/>
+      <c r="J11" s="19"/>
+      <c r="K11" s="31"/>
     </row>
     <row r="12" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="14" t="s">
@@ -2674,331 +2702,331 @@
       <c r="F12" s="15"/>
       <c r="G12" s="15"/>
       <c r="H12" s="15"/>
-      <c r="I12" s="23"/>
+      <c r="I12" s="22"/>
       <c r="J12" s="15"/>
-      <c r="K12" s="31"/>
+      <c r="K12" s="30"/>
     </row>
     <row r="13" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B13" s="17" t="s">
+      <c r="B13" s="18" t="s">
         <v>121</v>
       </c>
-      <c r="C13" s="18"/>
-      <c r="D13" s="18"/>
-      <c r="E13" s="18"/>
-      <c r="F13" s="18"/>
-      <c r="G13" s="18"/>
-      <c r="H13" s="18"/>
-      <c r="I13" s="23"/>
-      <c r="J13" s="18"/>
-      <c r="K13" s="32"/>
+      <c r="C13" s="19"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="19"/>
+      <c r="F13" s="19"/>
+      <c r="G13" s="19"/>
+      <c r="H13" s="19"/>
+      <c r="I13" s="22"/>
+      <c r="J13" s="19"/>
+      <c r="K13" s="31"/>
     </row>
     <row r="14" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B14" s="24" t="s">
+      <c r="B14" s="23" t="s">
         <v>122</v>
       </c>
-      <c r="C14" s="25"/>
-      <c r="D14" s="25"/>
-      <c r="E14" s="25"/>
-      <c r="F14" s="25"/>
-      <c r="G14" s="25"/>
-      <c r="H14" s="25"/>
-      <c r="I14" s="26"/>
-      <c r="J14" s="25"/>
-      <c r="K14" s="25"/>
+      <c r="C14" s="24"/>
+      <c r="D14" s="24"/>
+      <c r="E14" s="24"/>
+      <c r="F14" s="24"/>
+      <c r="G14" s="24"/>
+      <c r="H14" s="24"/>
+      <c r="I14" s="25"/>
+      <c r="J14" s="24"/>
+      <c r="K14" s="24"/>
     </row>
     <row r="15" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B15" s="27" t="s">
+      <c r="B15" s="26" t="s">
         <v>123</v>
       </c>
-      <c r="C15" s="28"/>
-      <c r="D15" s="28"/>
-      <c r="E15" s="28"/>
-      <c r="F15" s="28"/>
-      <c r="G15" s="28"/>
-      <c r="H15" s="28"/>
-      <c r="I15" s="26"/>
-      <c r="J15" s="28"/>
-      <c r="K15" s="28"/>
+      <c r="C15" s="27"/>
+      <c r="D15" s="27"/>
+      <c r="E15" s="27"/>
+      <c r="F15" s="27"/>
+      <c r="G15" s="27"/>
+      <c r="H15" s="27"/>
+      <c r="I15" s="25"/>
+      <c r="J15" s="27"/>
+      <c r="K15" s="27"/>
     </row>
     <row r="16" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B16" s="24" t="s">
+      <c r="B16" s="23" t="s">
         <v>124</v>
       </c>
-      <c r="C16" s="25"/>
-      <c r="D16" s="25"/>
-      <c r="E16" s="25"/>
-      <c r="F16" s="25"/>
-      <c r="G16" s="25"/>
-      <c r="H16" s="25"/>
-      <c r="I16" s="26"/>
-      <c r="J16" s="25"/>
-      <c r="K16" s="25"/>
+      <c r="C16" s="24"/>
+      <c r="D16" s="24"/>
+      <c r="E16" s="24"/>
+      <c r="F16" s="24"/>
+      <c r="G16" s="24"/>
+      <c r="H16" s="24"/>
+      <c r="I16" s="25"/>
+      <c r="J16" s="24"/>
+      <c r="K16" s="24"/>
     </row>
     <row r="17" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B17" s="27" t="s">
+      <c r="B17" s="26" t="s">
         <v>125</v>
       </c>
-      <c r="C17" s="28"/>
-      <c r="D17" s="28"/>
-      <c r="E17" s="28"/>
-      <c r="F17" s="28"/>
-      <c r="G17" s="28"/>
-      <c r="H17" s="28"/>
-      <c r="I17" s="26"/>
-      <c r="J17" s="28"/>
-      <c r="K17" s="28"/>
+      <c r="C17" s="27"/>
+      <c r="D17" s="27"/>
+      <c r="E17" s="27"/>
+      <c r="F17" s="27"/>
+      <c r="G17" s="27"/>
+      <c r="H17" s="27"/>
+      <c r="I17" s="25"/>
+      <c r="J17" s="27"/>
+      <c r="K17" s="27"/>
     </row>
     <row r="18" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B18" s="24" t="s">
+      <c r="B18" s="23" t="s">
         <v>126</v>
       </c>
-      <c r="C18" s="25"/>
-      <c r="D18" s="25"/>
-      <c r="E18" s="25"/>
-      <c r="F18" s="25"/>
-      <c r="G18" s="25"/>
-      <c r="H18" s="25"/>
-      <c r="I18" s="26"/>
-      <c r="J18" s="25"/>
-      <c r="K18" s="25"/>
+      <c r="C18" s="24"/>
+      <c r="D18" s="24"/>
+      <c r="E18" s="24"/>
+      <c r="F18" s="24"/>
+      <c r="G18" s="24"/>
+      <c r="H18" s="24"/>
+      <c r="I18" s="25"/>
+      <c r="J18" s="24"/>
+      <c r="K18" s="24"/>
     </row>
     <row r="19" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B19" s="27" t="s">
+      <c r="B19" s="26" t="s">
         <v>127</v>
       </c>
-      <c r="C19" s="28"/>
-      <c r="D19" s="28"/>
-      <c r="E19" s="28"/>
-      <c r="F19" s="28"/>
-      <c r="G19" s="28"/>
-      <c r="H19" s="28"/>
-      <c r="I19" s="26"/>
-      <c r="J19" s="28"/>
-      <c r="K19" s="28"/>
+      <c r="C19" s="27"/>
+      <c r="D19" s="27"/>
+      <c r="E19" s="27"/>
+      <c r="F19" s="27"/>
+      <c r="G19" s="27"/>
+      <c r="H19" s="27"/>
+      <c r="I19" s="25"/>
+      <c r="J19" s="27"/>
+      <c r="K19" s="27"/>
     </row>
     <row r="20" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B20" s="24" t="s">
+      <c r="B20" s="23" t="s">
         <v>128</v>
       </c>
-      <c r="C20" s="25"/>
-      <c r="D20" s="25"/>
-      <c r="E20" s="25"/>
-      <c r="F20" s="25"/>
-      <c r="G20" s="25"/>
-      <c r="H20" s="25"/>
-      <c r="I20" s="26"/>
-      <c r="J20" s="25"/>
-      <c r="K20" s="25"/>
+      <c r="C20" s="24"/>
+      <c r="D20" s="24"/>
+      <c r="E20" s="24"/>
+      <c r="F20" s="24"/>
+      <c r="G20" s="24"/>
+      <c r="H20" s="24"/>
+      <c r="I20" s="25"/>
+      <c r="J20" s="24"/>
+      <c r="K20" s="24"/>
     </row>
     <row r="21" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B21" s="27" t="s">
+      <c r="B21" s="26" t="s">
         <v>129</v>
       </c>
-      <c r="C21" s="28"/>
-      <c r="D21" s="28"/>
-      <c r="E21" s="28"/>
-      <c r="F21" s="28"/>
-      <c r="G21" s="28"/>
-      <c r="H21" s="28"/>
-      <c r="I21" s="26"/>
-      <c r="J21" s="28"/>
-      <c r="K21" s="28"/>
+      <c r="C21" s="27"/>
+      <c r="D21" s="27"/>
+      <c r="E21" s="27"/>
+      <c r="F21" s="27"/>
+      <c r="G21" s="27"/>
+      <c r="H21" s="27"/>
+      <c r="I21" s="25"/>
+      <c r="J21" s="27"/>
+      <c r="K21" s="27"/>
     </row>
     <row r="22" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B22" s="24" t="s">
+      <c r="B22" s="23" t="s">
         <v>130</v>
       </c>
-      <c r="C22" s="25"/>
-      <c r="D22" s="25"/>
-      <c r="E22" s="25"/>
-      <c r="F22" s="25"/>
-      <c r="G22" s="25"/>
-      <c r="H22" s="25"/>
-      <c r="I22" s="26"/>
-      <c r="J22" s="25"/>
-      <c r="K22" s="25"/>
+      <c r="C22" s="24"/>
+      <c r="D22" s="24"/>
+      <c r="E22" s="24"/>
+      <c r="F22" s="24"/>
+      <c r="G22" s="24"/>
+      <c r="H22" s="24"/>
+      <c r="I22" s="25"/>
+      <c r="J22" s="24"/>
+      <c r="K22" s="24"/>
     </row>
     <row r="23" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B23" s="27" t="s">
+      <c r="B23" s="26" t="s">
         <v>131</v>
       </c>
-      <c r="C23" s="28"/>
-      <c r="D23" s="28"/>
-      <c r="E23" s="28"/>
-      <c r="F23" s="28"/>
-      <c r="G23" s="28"/>
-      <c r="H23" s="28"/>
-      <c r="I23" s="26"/>
-      <c r="J23" s="28"/>
-      <c r="K23" s="28"/>
+      <c r="C23" s="27"/>
+      <c r="D23" s="27"/>
+      <c r="E23" s="27"/>
+      <c r="F23" s="27"/>
+      <c r="G23" s="27"/>
+      <c r="H23" s="27"/>
+      <c r="I23" s="25"/>
+      <c r="J23" s="27"/>
+      <c r="K23" s="27"/>
     </row>
     <row r="24" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B24" s="24" t="s">
+      <c r="B24" s="23" t="s">
         <v>132</v>
       </c>
-      <c r="C24" s="25"/>
-      <c r="D24" s="25"/>
-      <c r="E24" s="25"/>
-      <c r="F24" s="25"/>
-      <c r="G24" s="25"/>
-      <c r="H24" s="25"/>
-      <c r="I24" s="26"/>
-      <c r="J24" s="25"/>
-      <c r="K24" s="25"/>
+      <c r="C24" s="24"/>
+      <c r="D24" s="24"/>
+      <c r="E24" s="24"/>
+      <c r="F24" s="24"/>
+      <c r="G24" s="24"/>
+      <c r="H24" s="24"/>
+      <c r="I24" s="25"/>
+      <c r="J24" s="24"/>
+      <c r="K24" s="24"/>
     </row>
     <row r="25" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B25" s="27" t="s">
+      <c r="B25" s="26" t="s">
         <v>133</v>
       </c>
-      <c r="C25" s="28"/>
-      <c r="D25" s="28"/>
-      <c r="E25" s="28"/>
-      <c r="F25" s="28"/>
-      <c r="G25" s="28"/>
-      <c r="H25" s="28"/>
-      <c r="I25" s="26"/>
-      <c r="J25" s="28"/>
-      <c r="K25" s="28"/>
+      <c r="C25" s="27"/>
+      <c r="D25" s="27"/>
+      <c r="E25" s="27"/>
+      <c r="F25" s="27"/>
+      <c r="G25" s="27"/>
+      <c r="H25" s="27"/>
+      <c r="I25" s="25"/>
+      <c r="J25" s="27"/>
+      <c r="K25" s="27"/>
     </row>
     <row r="26" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B26" s="24" t="s">
+      <c r="B26" s="23" t="s">
         <v>134</v>
       </c>
-      <c r="C26" s="25"/>
-      <c r="D26" s="25"/>
-      <c r="E26" s="25"/>
-      <c r="F26" s="25"/>
-      <c r="G26" s="25"/>
-      <c r="H26" s="25"/>
-      <c r="I26" s="26"/>
-      <c r="J26" s="25"/>
-      <c r="K26" s="25"/>
+      <c r="C26" s="24"/>
+      <c r="D26" s="24"/>
+      <c r="E26" s="24"/>
+      <c r="F26" s="24"/>
+      <c r="G26" s="24"/>
+      <c r="H26" s="24"/>
+      <c r="I26" s="25"/>
+      <c r="J26" s="24"/>
+      <c r="K26" s="24"/>
     </row>
     <row r="27" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B27" s="27" t="s">
+      <c r="B27" s="26" t="s">
         <v>135</v>
       </c>
-      <c r="C27" s="28"/>
-      <c r="D27" s="28"/>
-      <c r="E27" s="28"/>
-      <c r="F27" s="28"/>
-      <c r="G27" s="28"/>
-      <c r="H27" s="28"/>
-      <c r="I27" s="26"/>
-      <c r="J27" s="28"/>
-      <c r="K27" s="28"/>
+      <c r="C27" s="27"/>
+      <c r="D27" s="27"/>
+      <c r="E27" s="27"/>
+      <c r="F27" s="27"/>
+      <c r="G27" s="27"/>
+      <c r="H27" s="27"/>
+      <c r="I27" s="25"/>
+      <c r="J27" s="27"/>
+      <c r="K27" s="27"/>
     </row>
     <row r="28" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B28" s="24" t="s">
+      <c r="B28" s="23" t="s">
         <v>136</v>
       </c>
-      <c r="C28" s="25"/>
-      <c r="D28" s="25"/>
-      <c r="E28" s="25"/>
-      <c r="F28" s="25"/>
-      <c r="G28" s="25"/>
-      <c r="H28" s="25"/>
-      <c r="I28" s="26"/>
-      <c r="J28" s="25"/>
-      <c r="K28" s="25"/>
+      <c r="C28" s="24"/>
+      <c r="D28" s="24"/>
+      <c r="E28" s="24"/>
+      <c r="F28" s="24"/>
+      <c r="G28" s="24"/>
+      <c r="H28" s="24"/>
+      <c r="I28" s="25"/>
+      <c r="J28" s="24"/>
+      <c r="K28" s="24"/>
     </row>
     <row r="29" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B29" s="27" t="s">
+      <c r="B29" s="26" t="s">
         <v>137</v>
       </c>
-      <c r="C29" s="28"/>
-      <c r="D29" s="28"/>
-      <c r="E29" s="28"/>
-      <c r="F29" s="28"/>
-      <c r="G29" s="28"/>
-      <c r="H29" s="28"/>
-      <c r="I29" s="26"/>
-      <c r="J29" s="28"/>
-      <c r="K29" s="28"/>
+      <c r="C29" s="27"/>
+      <c r="D29" s="27"/>
+      <c r="E29" s="27"/>
+      <c r="F29" s="27"/>
+      <c r="G29" s="27"/>
+      <c r="H29" s="27"/>
+      <c r="I29" s="25"/>
+      <c r="J29" s="27"/>
+      <c r="K29" s="27"/>
     </row>
     <row r="30" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B30" s="24" t="s">
+      <c r="B30" s="23" t="s">
         <v>138</v>
       </c>
-      <c r="C30" s="25"/>
-      <c r="D30" s="25"/>
-      <c r="E30" s="25"/>
-      <c r="F30" s="25"/>
-      <c r="G30" s="25"/>
-      <c r="H30" s="25"/>
-      <c r="I30" s="26"/>
-      <c r="J30" s="25"/>
-      <c r="K30" s="25"/>
+      <c r="C30" s="24"/>
+      <c r="D30" s="24"/>
+      <c r="E30" s="24"/>
+      <c r="F30" s="24"/>
+      <c r="G30" s="24"/>
+      <c r="H30" s="24"/>
+      <c r="I30" s="25"/>
+      <c r="J30" s="24"/>
+      <c r="K30" s="24"/>
     </row>
     <row r="31" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B31" s="27" t="s">
+      <c r="B31" s="26" t="s">
         <v>139</v>
       </c>
-      <c r="C31" s="28"/>
-      <c r="D31" s="28"/>
-      <c r="E31" s="28"/>
-      <c r="F31" s="28"/>
-      <c r="G31" s="28"/>
-      <c r="H31" s="28"/>
-      <c r="I31" s="26"/>
-      <c r="J31" s="28"/>
-      <c r="K31" s="28"/>
+      <c r="C31" s="27"/>
+      <c r="D31" s="27"/>
+      <c r="E31" s="27"/>
+      <c r="F31" s="27"/>
+      <c r="G31" s="27"/>
+      <c r="H31" s="27"/>
+      <c r="I31" s="25"/>
+      <c r="J31" s="27"/>
+      <c r="K31" s="27"/>
     </row>
     <row r="32" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B32" s="24" t="s">
+      <c r="B32" s="23" t="s">
         <v>140</v>
       </c>
-      <c r="C32" s="25"/>
-      <c r="D32" s="25"/>
-      <c r="E32" s="25"/>
-      <c r="F32" s="25"/>
-      <c r="G32" s="25"/>
-      <c r="H32" s="25"/>
-      <c r="I32" s="26"/>
-      <c r="J32" s="25"/>
-      <c r="K32" s="25"/>
+      <c r="C32" s="24"/>
+      <c r="D32" s="24"/>
+      <c r="E32" s="24"/>
+      <c r="F32" s="24"/>
+      <c r="G32" s="24"/>
+      <c r="H32" s="24"/>
+      <c r="I32" s="25"/>
+      <c r="J32" s="24"/>
+      <c r="K32" s="24"/>
     </row>
     <row r="33" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B33" s="27" t="s">
+      <c r="B33" s="26" t="s">
         <v>141</v>
       </c>
-      <c r="C33" s="28"/>
-      <c r="D33" s="28"/>
-      <c r="E33" s="28"/>
-      <c r="F33" s="28"/>
-      <c r="G33" s="28"/>
-      <c r="H33" s="28"/>
-      <c r="I33" s="26"/>
-      <c r="J33" s="28"/>
-      <c r="K33" s="28"/>
+      <c r="C33" s="27"/>
+      <c r="D33" s="27"/>
+      <c r="E33" s="27"/>
+      <c r="F33" s="27"/>
+      <c r="G33" s="27"/>
+      <c r="H33" s="27"/>
+      <c r="I33" s="25"/>
+      <c r="J33" s="27"/>
+      <c r="K33" s="27"/>
     </row>
     <row r="34" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B34" s="24" t="s">
+      <c r="B34" s="23" t="s">
         <v>142</v>
       </c>
-      <c r="C34" s="25"/>
-      <c r="D34" s="25"/>
-      <c r="E34" s="25"/>
-      <c r="F34" s="25"/>
-      <c r="G34" s="25"/>
-      <c r="H34" s="25"/>
-      <c r="I34" s="26"/>
-      <c r="J34" s="25"/>
-      <c r="K34" s="25"/>
+      <c r="C34" s="24"/>
+      <c r="D34" s="24"/>
+      <c r="E34" s="24"/>
+      <c r="F34" s="24"/>
+      <c r="G34" s="24"/>
+      <c r="H34" s="24"/>
+      <c r="I34" s="25"/>
+      <c r="J34" s="24"/>
+      <c r="K34" s="24"/>
     </row>
     <row r="35" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B35" s="27" t="s">
+      <c r="B35" s="26" t="s">
         <v>143</v>
       </c>
-      <c r="C35" s="28"/>
-      <c r="D35" s="28"/>
-      <c r="E35" s="28"/>
-      <c r="F35" s="28"/>
-      <c r="G35" s="28"/>
-      <c r="H35" s="28"/>
-      <c r="I35" s="26"/>
-      <c r="J35" s="28"/>
-      <c r="K35" s="28"/>
+      <c r="C35" s="27"/>
+      <c r="D35" s="27"/>
+      <c r="E35" s="27"/>
+      <c r="F35" s="27"/>
+      <c r="G35" s="27"/>
+      <c r="H35" s="27"/>
+      <c r="I35" s="25"/>
+      <c r="J35" s="27"/>
+      <c r="K35" s="27"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -3033,138 +3061,141 @@
   </cols>
   <sheetData>
     <row r="2" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="9" t="s">
         <v>144</v>
       </c>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
     </row>
     <row r="4" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B4" s="34" t="s">
+      <c r="B4" s="33" t="s">
         <v>145</v>
       </c>
-      <c r="C4" s="34"/>
-      <c r="D4" s="34"/>
-      <c r="E4" s="34"/>
+      <c r="C4" s="33"/>
+      <c r="D4" s="33"/>
+      <c r="E4" s="33"/>
     </row>
     <row r="6" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B6" s="35" t="s">
+      <c r="B6" s="34" t="s">
         <v>146</v>
       </c>
-      <c r="C6" s="36" t="n">
+      <c r="C6" s="35" t="n">
         <f aca="false">COUNTA('🖥 HARDWARE'!C6:C50)</f>
         <v>0</v>
       </c>
-      <c r="D6" s="36"/>
-      <c r="E6" s="36"/>
+      <c r="D6" s="35"/>
+      <c r="E6" s="35"/>
     </row>
     <row r="7" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B7" s="35" t="s">
+      <c r="B7" s="34" t="s">
         <v>147</v>
       </c>
-      <c r="C7" s="36" t="n">
+      <c r="C7" s="35" t="n">
         <f aca="false">COUNTA('💾 SOFTWARE'!C6:C50)</f>
         <v>0</v>
       </c>
-      <c r="D7" s="36"/>
-      <c r="E7" s="36"/>
+      <c r="D7" s="35"/>
+      <c r="E7" s="35"/>
     </row>
     <row r="8" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B8" s="35" t="s">
+      <c r="B8" s="34" t="s">
         <v>148</v>
       </c>
-      <c r="C8" s="36" t="n">
+      <c r="C8" s="35" t="n">
         <f aca="false">COUNTA('☁️ CLOUD E SAAS'!C6:C50)</f>
         <v>0</v>
       </c>
-      <c r="D8" s="36"/>
-      <c r="E8" s="36"/>
+      <c r="D8" s="35"/>
+      <c r="E8" s="35"/>
     </row>
     <row r="9" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B9" s="35" t="s">
+      <c r="B9" s="34" t="s">
         <v>149</v>
       </c>
-      <c r="C9" s="36" t="n">
+      <c r="C9" s="35" t="n">
         <f aca="false">COUNTA('🌐 SUPERFÍCIE EXTERNA'!C6:C50)</f>
         <v>0</v>
       </c>
+      <c r="D9" s="35"/>
+      <c r="E9" s="35"/>
     </row>
     <row r="10" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B10" s="37" t="s">
+      <c r="B10" s="36" t="s">
         <v>150</v>
       </c>
-      <c r="C10" s="37"/>
-      <c r="D10" s="37"/>
-      <c r="E10" s="37"/>
+      <c r="C10" s="36"/>
+      <c r="D10" s="36"/>
+      <c r="E10" s="36"/>
     </row>
     <row r="12" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B12" s="38" t="s">
+      <c r="B12" s="37" t="s">
         <v>151</v>
       </c>
-      <c r="C12" s="39" t="n">
-        <f aca="false">COUNTIF('🖥 HARDWARE'!I6:I50,"🔴 CRÍTICO")</f>
+      <c r="C12" s="38" t="n">
+        <f aca="false">COUNTIF('🖥 HARDWARE'!I6:I50,"*CRÍTICO*")</f>
         <v>0</v>
       </c>
-      <c r="D12" s="39"/>
-      <c r="E12" s="39"/>
+      <c r="D12" s="38"/>
+      <c r="E12" s="38"/>
     </row>
     <row r="13" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B13" s="40" t="s">
+      <c r="B13" s="39" t="s">
         <v>152</v>
       </c>
-      <c r="C13" s="41" t="n">
-        <f aca="false">COUNTIF('🖥 HARDWARE'!I6:I50,"🟠 ALTO")</f>
+      <c r="C13" s="40" t="n">
+        <f aca="false">COUNTIF('🖥 HARDWARE'!I6:I50,"*ALTO*")</f>
         <v>0</v>
       </c>
-      <c r="D13" s="41"/>
-      <c r="E13" s="41"/>
+      <c r="D13" s="40"/>
+      <c r="E13" s="40"/>
     </row>
     <row r="14" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B14" s="42" t="s">
+      <c r="B14" s="41" t="s">
         <v>153</v>
       </c>
-      <c r="C14" s="43" t="n">
-        <f aca="false">COUNTIF('🖥 HARDWARE'!I6:I50,"🟡 MÉDIO")</f>
+      <c r="C14" s="42" t="n">
+        <f aca="false">COUNTIF('🖥 HARDWARE'!I6:I50,"*MÉDIO*")</f>
         <v>0</v>
       </c>
-      <c r="D14" s="43"/>
-      <c r="E14" s="43"/>
+      <c r="D14" s="42"/>
+      <c r="E14" s="42"/>
     </row>
     <row r="16" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B16" s="44" t="s">
+      <c r="B16" s="43" t="s">
         <v>154</v>
       </c>
-      <c r="C16" s="44"/>
-      <c r="D16" s="44"/>
-      <c r="E16" s="44"/>
+      <c r="C16" s="43"/>
+      <c r="D16" s="43"/>
+      <c r="E16" s="43"/>
     </row>
     <row r="18" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B18" s="38" t="s">
+      <c r="B18" s="37" t="s">
         <v>155</v>
       </c>
-      <c r="C18" s="39" t="n">
+      <c r="C18" s="38" t="n">
         <f aca="false">COUNTIF('☁️ CLOUD E SAAS'!K6:K50,"❌*")</f>
         <v>0</v>
       </c>
-      <c r="D18" s="39"/>
-      <c r="E18" s="39"/>
+      <c r="D18" s="38"/>
+      <c r="E18" s="38"/>
     </row>
     <row r="20" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B20" s="45" t="s">
+      <c r="B20" s="44" t="s">
         <v>156</v>
       </c>
-      <c r="C20" s="45"/>
-      <c r="D20" s="45"/>
-      <c r="E20" s="45"/>
+      <c r="C20" s="44"/>
+      <c r="D20" s="44"/>
+      <c r="E20" s="44"/>
     </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="13">
     <mergeCell ref="B2:E2"/>
     <mergeCell ref="B4:E4"/>
     <mergeCell ref="C6:E6"/>
     <mergeCell ref="C7:E7"/>
     <mergeCell ref="C8:E8"/>
+    <mergeCell ref="C9:E9"/>
     <mergeCell ref="B10:E10"/>
     <mergeCell ref="C12:E12"/>
     <mergeCell ref="C13:E13"/>

</xml_diff>